<commit_message>
Add Battery Detail (DALA+CAN) and Force Charge mode
</commit_message>
<xml_diff>
--- a/Dovecote_StartupLoan_CashFlow_SurvivalBudget.xlsx
+++ b/Dovecote_StartupLoan_CashFlow_SurvivalBudget.xlsx
@@ -132,7 +132,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -154,11 +154,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -247,6 +291,10 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -656,7 +704,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.075</v>
+        <v>0.06</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -685,12 +733,12 @@
           <t>Monthly repayment</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>501</v>
+      <c r="B8" s="4" t="n">
+        <v>483</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>£ (approx — 7.5% over 5 yrs)</t>
+          <t>£/mo (approx — 6% over 5 yrs, interest-only Year 1 = £125/mo)</t>
         </is>
       </c>
     </row>
@@ -725,107 +773,122 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1"/>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>HV electrical commissioning (Node-3)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>£ — Month 1</t>
-        </is>
-      </c>
-    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ASIC mining net revenue (Z15, after electricity)</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="n">
+        <v>446</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>£/mo (£5,351/yr net — gross £7,322 minus £1,971 electricity at 15p/kWh)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1"/>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Public liability insurance</t>
+          <t>HV electrical commissioning (Node-3)</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>£/yr — Month 1</t>
+          <t>£ — Month 1</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Private electrician training — full JIB Gold Card programme</t>
+          <t>Public liability insurance</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>9000</v>
+        <v>800</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>£ — Month 1 (18-month programme)</t>
+          <t>£/yr — Month 1</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Director's loan reimbursement (inverter £1,200 + batteries £1,800 + trailer £800)</t>
+          <t>Private electrician training — full JIB Gold Card programme</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>3800</v>
+        <v>9000</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>£ — Month 1</t>
+          <t>£ — Month 1 (18-month programme)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Company van HP deposit (10% of £8,000)</t>
+          <t>Director's loan reimbursement (inverter £1,200 + batteries £1,800 + trailer £800)</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>800</v>
+        <v>3800</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>£ — Month 1. Matt's loan. Van is company asset.</t>
+          <t>£ — Month 1</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Company van HP monthly payment (~7% APR, 4yr)</t>
+          <t>Company van HP deposit (10% of £8,000)</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>175</v>
+        <v>800</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>£/mo from Month 2. Matt's loan.</t>
+          <t>£ — Month 1. Matt's loan. Van is company asset.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Company van HP monthly payment (~7% APR, 4yr)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>£/mo from Month 2. Matt's loan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Working capital reserve (held in account)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B20" s="4" t="n">
         <v>8600</v>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>£ — implicit in closing balance (£9,400 less £800 van deposit)</t>
         </is>
@@ -846,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -874,7 +937,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Matt Brander — Start Up Loan Application | Company No. 17160178 | £25,000 at 7.5% over 5 years</t>
+          <t>Matt Brander — Start Up Loan Application | Company No. 17160178 | £25,000 at 6% over 5 years</t>
         </is>
       </c>
     </row>
@@ -1126,106 +1189,106 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ASIC mining — Z15 (net after electricity, from Month 3)</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="H10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="J10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="K10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="L10" s="35" t="n">
+        <v>446</v>
+      </c>
+      <c r="M10" s="35" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>TOTAL INCOME</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B11" t="n">
         <v>25000</v>
       </c>
-      <c r="C10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <v>150</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <v>199</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>199</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="I10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="J10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="K10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="L10" s="18" t="n">
-        <v>461</v>
-      </c>
-      <c r="M10" s="18" t="n">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>596</v>
+      </c>
+      <c r="E11" t="n">
+        <v>645</v>
+      </c>
+      <c r="F11" t="n">
+        <v>645</v>
+      </c>
+      <c r="G11" t="n">
+        <v>907</v>
+      </c>
+      <c r="H11" t="n">
+        <v>907</v>
+      </c>
+      <c r="I11" t="n">
+        <v>907</v>
+      </c>
+      <c r="J11" t="n">
+        <v>907</v>
+      </c>
+      <c r="K11" t="n">
+        <v>907</v>
+      </c>
+      <c r="L11" t="n">
+        <v>907</v>
+      </c>
+      <c r="M11" t="n">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>EXPENDITURE</t>
         </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>HV electrical commissioning — Node-3</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="16" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Public liability insurance</t>
+          <t>HV electrical commissioning — Node-3</t>
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>0</v>
@@ -1264,11 +1327,11 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Private electrician training — JIB Gold Card programme</t>
+          <t>Public liability insurance</t>
         </is>
       </c>
       <c r="B14" s="16" t="n">
-        <v>9000</v>
+        <v>800</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>0</v>
@@ -1307,11 +1370,11 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Director's loan reimbursement (inverter + batteries + trailer)</t>
+          <t>Private electrician training — JIB Gold Card programme</t>
         </is>
       </c>
       <c r="B15" s="16" t="n">
-        <v>3800</v>
+        <v>9000</v>
       </c>
       <c r="C15" s="16" t="n">
         <v>0</v>
@@ -1350,11 +1413,11 @@
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Company van — hire purchase deposit (10% of £8,000)</t>
+          <t>Director's loan reimbursement (inverter + batteries + trailer)</t>
         </is>
       </c>
       <c r="B16" s="16" t="n">
-        <v>800</v>
+        <v>3800</v>
       </c>
       <c r="C16" s="16" t="n">
         <v>0</v>
@@ -1393,282 +1456,301 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
+          <t>Company van — hire purchase deposit (10% of £8,000)</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
           <t>Company van — hire purchase payments (~7% APR, 4 years)</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="16" t="n">
+      <c r="B18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="G17" s="16" t="n">
+      <c r="G18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="H17" s="16" t="n">
+      <c r="H18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="I17" s="16" t="n">
+      <c r="I18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="J17" s="16" t="n">
+      <c r="J18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="K17" s="16" t="n">
+      <c r="K18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="L17" s="16" t="n">
+      <c r="L18" s="16" t="n">
         <v>175</v>
       </c>
-      <c r="M17" s="16" t="n">
+      <c r="M18" s="16" t="n">
         <v>175</v>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Loan repayment — £501/mo from Month 2</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="D18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="E18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="F18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="G18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="H18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="I18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="J18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="K18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="L18" s="21" t="n">
-        <v>501</v>
-      </c>
-      <c r="M18" s="21" t="n">
-        <v>501</v>
-      </c>
-    </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Loan repayment — £125/mo interest only (12-month capital repayment holiday). Full £483/mo from Month 13.</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="G19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="H19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="I19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="J19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="K19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="M19" s="21" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>TOTAL EXPENDITURE</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
-        <v>16400</v>
-      </c>
-      <c r="C19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="D19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="E19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="F19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="G19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="H19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="I19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="J19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="K19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>676</v>
-      </c>
-      <c r="M19" s="23" t="n">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="36" t="n"/>
+      <c r="D20" s="36" t="n"/>
+      <c r="E20" s="36" t="n"/>
+      <c r="F20" s="36" t="n"/>
+      <c r="G20" s="36" t="n"/>
+      <c r="H20" s="36" t="n"/>
+      <c r="I20" s="36" t="n"/>
+      <c r="J20" s="36" t="n"/>
+      <c r="K20" s="36" t="n"/>
+      <c r="L20" s="36" t="n"/>
+      <c r="M20" s="36" t="n"/>
+      <c r="N20" s="37" t="n"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>CASH POSITION (Working capital buffer visible in closing balance)</t>
         </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Net cash flow (month)</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="n">
-        <v>8600</v>
-      </c>
-      <c r="C21" s="16" t="n">
-        <v>-676</v>
-      </c>
-      <c r="D21" s="16" t="n">
-        <v>-526</v>
-      </c>
-      <c r="E21" s="16" t="n">
-        <v>-477</v>
-      </c>
-      <c r="F21" s="16" t="n">
-        <v>-477</v>
-      </c>
-      <c r="G21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="H21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="I21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="J21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="K21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="L21" s="16" t="n">
-        <v>-215</v>
-      </c>
-      <c r="M21" s="16" t="n">
-        <v>-215</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
+          <t>Net cash flow (month)</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>8600</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>-676</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <v>-80</v>
+      </c>
+      <c r="E22" s="16" t="n">
+        <v>-31</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>-31</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="I22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="J22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="K22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="L22" s="16" t="n">
+        <v>231</v>
+      </c>
+      <c r="M22" s="16" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
           <t>Opening balance</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="16" t="n">
+      <c r="B23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="16" t="n">
         <v>8600</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D23" s="16" t="n">
         <v>7924</v>
       </c>
-      <c r="E22" s="16" t="n">
-        <v>7398</v>
-      </c>
-      <c r="F22" s="16" t="n">
-        <v>6921</v>
-      </c>
-      <c r="G22" s="16" t="n">
-        <v>6444</v>
-      </c>
-      <c r="H22" s="16" t="n">
-        <v>6229</v>
-      </c>
-      <c r="I22" s="16" t="n">
-        <v>6014</v>
-      </c>
-      <c r="J22" s="16" t="n">
-        <v>5799</v>
-      </c>
-      <c r="K22" s="16" t="n">
-        <v>5584</v>
-      </c>
-      <c r="L22" s="16" t="n">
-        <v>5369</v>
-      </c>
-      <c r="M22" s="16" t="n">
-        <v>5154</v>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="E23" s="16" t="n">
+        <v>7844</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>7813</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>7782</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>8013</v>
+      </c>
+      <c r="I23" s="16" t="n">
+        <v>8244</v>
+      </c>
+      <c r="J23" s="16" t="n">
+        <v>8475</v>
+      </c>
+      <c r="K23" s="16" t="n">
+        <v>8706</v>
+      </c>
+      <c r="L23" s="16" t="n">
+        <v>8937</v>
+      </c>
+      <c r="M23" s="16" t="n">
+        <v>9168</v>
+      </c>
+    </row>
+    <row r="24" ht="8" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>CLOSING BALANCE</t>
         </is>
       </c>
-      <c r="B23" s="25" t="n">
+      <c r="B24" s="25" t="n">
         <v>8600</v>
       </c>
-      <c r="C23" s="25" t="n">
+      <c r="C24" s="25" t="n">
         <v>7924</v>
       </c>
-      <c r="D23" s="25" t="n">
-        <v>7398</v>
-      </c>
-      <c r="E23" s="25" t="n">
-        <v>6921</v>
-      </c>
-      <c r="F23" s="25" t="n">
-        <v>6444</v>
-      </c>
-      <c r="G23" s="25" t="n">
-        <v>6229</v>
-      </c>
-      <c r="H23" s="25" t="n">
-        <v>6014</v>
-      </c>
-      <c r="I23" s="25" t="n">
-        <v>5799</v>
-      </c>
-      <c r="J23" s="25" t="n">
-        <v>5584</v>
-      </c>
-      <c r="K23" s="25" t="n">
-        <v>5369</v>
-      </c>
-      <c r="L23" s="25" t="n">
-        <v>5154</v>
-      </c>
-      <c r="M23" s="25" t="n">
-        <v>4939</v>
-      </c>
-    </row>
-    <row r="24" ht="8" customHeight="1"/>
-    <row r="25" ht="72" customHeight="1">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t>Notes: Loan drawn in Month 1. Immediate deployment: HV commissioning £2,000, insurance £800, private electrician training (JIB Gold Card programme) £9,000, director's loan reimbursement (inverter £1,200 + batteries £1,800 + trailer £800) £3,800. Total deployed M1: £15,600. Remaining £9,400 held as working capital buffer. Node-3 Agile arbitrage (~£1,800/yr) from Month 3; StorageSub/algorithm licence: 1 subscriber per node at £49/mo — 1 sub from Month 4 (Node-3); Flexibility/BM revenue (£262/mo) from Month 6. StorageSub scales with fleet: 4 nodes by Year 2 = 4 subscribers = £196/mo. Full Year 2 run rate: £608/mo (£7,296/yr). Loan repayment £501/mo from Month 2. Personal redundancy settlement (~£22k net, Oct 2026) provides additional buffer not shown here.</t>
+      <c r="D24" s="25" t="n">
+        <v>7844</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>7813</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>7782</v>
+      </c>
+      <c r="G24" s="25" t="n">
+        <v>8013</v>
+      </c>
+      <c r="H24" s="25" t="n">
+        <v>8244</v>
+      </c>
+      <c r="I24" s="25" t="n">
+        <v>8475</v>
+      </c>
+      <c r="J24" s="25" t="n">
+        <v>8706</v>
+      </c>
+      <c r="K24" s="25" t="n">
+        <v>8937</v>
+      </c>
+      <c r="L24" s="25" t="n">
+        <v>9168</v>
+      </c>
+      <c r="M24" s="25" t="n">
+        <v>9399</v>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1"/>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>Notes: Loan drawn in Month 1. Immediate deployment: HV commissioning £2,000, insurance £800, private electrician training (JIB Gold Card programme) £9,000, director's loan reimbursement (inverter £1,200 + batteries £1,800 + trailer £800) £3,800. Total deployed M1: £15,600. Remaining £9,400 held as working capital buffer. Node-3 Agile arbitrage (~£1,800/yr) from Month 3; StorageSub/algorithm licence: 1 subscriber per node at £49/mo — 1 sub from Month 4 (Node-3); Flexibility/BM revenue (£262/mo) from Month 6. StorageSub scales with fleet: 4 nodes by Year 2 = 4 subscribers = £196/mo. Full Year 2 run rate: £608/mo (£7,296/yr). Loan repayment £125/mo interest only (12-month capital repayment holiday). Full £483/mo from Month 13.. Personal redundancy settlement (~£22k net, Oct 2026) provides additional buffer not shown here.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="5">
     <mergeCell ref="A20:N20"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A25:N25"/>
-    <mergeCell ref="A11:N11"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -1682,7 +1764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1700,7 +1782,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Complete the 'Monthly Amount (£)' column before submission. All figures are personal (not business).</t>
+          <t>Personal financial position — Matt Brander. Post-employment (from 24 Oct 2026). Income comprises COT3 settlement bridge drawdown and Dovecote director wages. Verify living cost figures before submission.</t>
         </is>
       </c>
     </row>
@@ -1736,23 +1818,27 @@
           <t>Employment income (until Oct 2026)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n"/>
+      <c r="B6" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>Ending 24 Oct — enter monthly net</t>
+          <t>NHS employment ends 24 Oct 2026. Zero from Nov 2026 onward.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="30" t="inlineStr">
         <is>
-          <t>Redundancy / termination payment</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="n"/>
+          <t>COT3 settlement payment (personal bridge drawdown)</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>1400</v>
+      </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>~£28k gross / ~£20-22k net — enter actual</t>
+          <t>COT3 settlement (Brander v UHS, Sept 2026). Gross £28,000 (PILON + holiday, taxable). Est. net £18,000–£20,000. £12,000 retained personally as bridge; £6,000 as director loan to Dovecote (3 miners). Additional £3,800 existing director loan owed by Dovecote repaid from revenue = £15,800 effective bridge (~10 months at £1,500/month).</t>
         </is>
       </c>
     </row>
@@ -1762,10 +1848,12 @@
           <t>Business income (Dovecote Systems)</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n"/>
+      <c r="B8" s="16" t="n">
+        <v>900</v>
+      </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>From cashflow forecast — enter as received</t>
+          <t>Director wage £900/mo from Month 3 (Nov 2026). Increases as node fleet scales.</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1863,9 @@
           <t>Other income</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n"/>
+      <c r="B9" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="C9" s="29" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1785,7 +1875,7 @@
         </is>
       </c>
       <c r="B10" s="18">
-        <f>SUM(B5:B9)</f>
+        <f>SUM(B6:B9)</f>
         <v/>
       </c>
       <c r="C10" s="29" t="inlineStr"/>
@@ -1810,8 +1900,14 @@
           <t>Mortgage / rent</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="29" t="inlineStr"/>
+      <c r="B13" s="16" t="n">
+        <v>400</v>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Shared accommodation — indicative. Verify actual figure.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
@@ -1819,7 +1915,9 @@
           <t>Council tax</t>
         </is>
       </c>
-      <c r="B14" s="16" t="n"/>
+      <c r="B14" s="16" t="n">
+        <v>120</v>
+      </c>
       <c r="C14" s="29" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -1828,7 +1926,9 @@
           <t>Utilities (gas, electric, water)</t>
         </is>
       </c>
-      <c r="B15" s="16" t="n"/>
+      <c r="B15" s="16" t="n">
+        <v>150</v>
+      </c>
       <c r="C15" s="29" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
@@ -1837,7 +1937,9 @@
           <t>Food &amp; groceries</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n"/>
+      <c r="B16" s="16" t="n">
+        <v>350</v>
+      </c>
       <c r="C16" s="29" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
@@ -1846,7 +1948,9 @@
           <t>Transport (fuel, insurance, MOT)</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n"/>
+      <c r="B17" s="16" t="n">
+        <v>200</v>
+      </c>
       <c r="C17" s="29" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -1855,7 +1959,9 @@
           <t>Mobile phone</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n"/>
+      <c r="B18" s="16" t="n">
+        <v>50</v>
+      </c>
       <c r="C18" s="29" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -1864,7 +1970,9 @@
           <t>Broadband / TV</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
+      <c r="B19" s="16" t="n">
+        <v>40</v>
+      </c>
       <c r="C19" s="29" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -1873,7 +1981,9 @@
           <t>Insurance (personal — home, life, etc.)</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n"/>
+      <c r="B20" s="16" t="n">
+        <v>50</v>
+      </c>
       <c r="C20" s="29" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -1882,7 +1992,9 @@
           <t>Clothing</t>
         </is>
       </c>
-      <c r="B21" s="16" t="n"/>
+      <c r="B21" s="16" t="n">
+        <v>30</v>
+      </c>
       <c r="C21" s="29" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -1891,7 +2003,9 @@
           <t>Subscriptions &amp; entertainment</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n"/>
+      <c r="B22" s="16" t="n">
+        <v>50</v>
+      </c>
       <c r="C22" s="29" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -1900,54 +2014,71 @@
           <t>Other regular expenses</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n"/>
+      <c r="B23" s="16" t="n">
+        <v>0</v>
+      </c>
       <c r="C23" s="29" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Existing unsecured debt repayments (cards &amp; loans — all current, no missed payments)</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>£57k unsecured debt (50% credit cards / 50% personal loans). All payments current. No defaults or missed payments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>Loan repayment (Start Up Loan)</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
-        <v>501</v>
-      </c>
-      <c r="C24" s="29" t="inlineStr">
-        <is>
-          <t>£501/mo fixed</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="B25" s="16" t="n">
+        <v>156</v>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>£156/month Year 1 (interest-only holiday at 7.5% p.a.). £501/month from Month 13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>TOTAL MONTHLY EXPENDITURE</t>
         </is>
       </c>
-      <c r="B25" s="23">
-        <f>SUM(B12:B27)</f>
+      <c r="B26" s="23">
+        <f>SUM(B13:B25)</f>
         <v/>
       </c>
-      <c r="C25" s="29" t="inlineStr"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="30" t="inlineStr"/>
-      <c r="B26" s="16" t="n"/>
       <c r="C26" s="29" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="33" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="29" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>MONTHLY SURPLUS / DEFICIT</t>
         </is>
       </c>
-      <c r="B27" s="21">
-        <f>B10-B28</f>
+      <c r="B28" s="21">
+        <f>B10-B26</f>
         <v/>
       </c>
-      <c r="C27" s="29" t="inlineStr">
-        <is>
-          <t>Must be positive or explain how covered</t>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Positive = surplus. Redundancy bridge covers shortfall while business ramps to 8+ nodes.</t>
         </is>
       </c>
     </row>

</xml_diff>